<commit_message>
Add Runtime sheet to analysis exporter
Per-config runtime mean/std/min/max plus a relative-to-fastest column,
with a hardware-comparability note. runtime_s has been recorded per seed
since P0 (sampling incl. ACO/SA search + final model fit).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/analysis/P1_rekap.xlsx
+++ b/results/analysis/P1_rekap.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agregat" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semua run" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semua run" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +41,11 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -82,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -90,6 +96,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1446,6 +1453,642 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Runtime per konfigurasi (detik per seed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>fitness_fn</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>stratified</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>replacement</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>seeds</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>runtime_mean_s</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>runtime_std_s</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>runtime_min_s</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>runtime_max_s</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>relatif_thd_tercepat</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>shs-aco-smote</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>gb</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>1149</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>6371.854</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>1117.1118</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>5154.67</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>7645.33</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>shs-aco-smote</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>gb</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1149</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>6598.308</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>623.7912</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>5528.04</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>7034.46</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>shs-aco-smote</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>gb</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>1149</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>6609.408</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>584.2399</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>5600.42</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>7077.23</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>shs-aco-smote</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>gb</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>1149</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>6660.86</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>566.3022</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>5679.79</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>7089.77</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>shs-aco-smote</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>gb</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1149</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>gmean</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>6727.112</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>633.9659</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>5915.73</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>7457.74</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>shs-aco-smote</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>gb</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>1149</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>6802.136</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>1220.2258</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>5500.09</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>8113.72</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>shs-aco-smote</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>gb</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1149</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>bas</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>7054.254</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>277.5559</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>6615.13</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>7343.48</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>shs-aco-smote</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>gb</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>1149</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>7059.552</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>364.8781</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>6514.03</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>7396.72</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>shs-aco-smote</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>gb</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>1149</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>7212.782</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>1029.2723</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>5396.41</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>7922.5</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>shs-aco-smote</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>gb</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>1149</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>7248.854</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>447.3228</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>6486.33</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>7629.06</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Catatan: runtime = sampling (termasuk pencarian ACO/SA) + pelatihan model final. Bandingkan hanya antar run pada mesin yang sama (P0 = MacBook M3; P1/P2 = Hetzner CPX42; 8 worker paralel berbagi core).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:S51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>